<commit_message>
ertrag korrigiert um zinsen pro quartal
</commit_message>
<xml_diff>
--- a/klas/erbschaft/nachlass/Nachlass_klas_krueger.xlsx
+++ b/klas/erbschaft/nachlass/Nachlass_klas_krueger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bk\bk_shared\klas\erbschaft\nachlass\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D6C4B3F170A4B06DDBCE5B378F82F9B35D00F821" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBB85D7-CA7B-4B4F-B36E-8BCC511794A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8760" yWindow="270" windowWidth="28800" windowHeight="14370" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="10410" windowWidth="38400" windowHeight="10470" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nachlassverzeichnis" sheetId="1" r:id="rId1"/>
@@ -31,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="55">
   <si>
     <t>Nachlasssache Klas Krüger</t>
   </si>
@@ -62,24 +59,7 @@
     <t>Depot comdirect 118 728563800, sonstiges</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Geschäftseinlage green-planetengergy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>5258263660</t>
-    </r>
+    <t>Geschäftseinlage green-planetengergy 5258263660</t>
   </si>
   <si>
     <t>50% LZO Konto</t>
@@ -100,6 +80,9 @@
     <t>comdirect Depot</t>
   </si>
   <si>
+    <t>(aus Blatt 'Ertrag comdirect 2025', korrigiert 20.10.2026)</t>
+  </si>
+  <si>
     <t>Erträge 2025 gesamt</t>
   </si>
   <si>
@@ -175,16 +158,40 @@
     <t>Depot</t>
   </si>
   <si>
-    <t xml:space="preserve">Ertragsgutschrift </t>
-  </si>
-  <si>
-    <t>Storno Ertragsgutschrift</t>
-  </si>
-  <si>
-    <t>Zinsen</t>
-  </si>
-  <si>
-    <t>Übertrag</t>
+    <t>Zinsen Tagesgeld Q1 (netto)</t>
+  </si>
+  <si>
+    <t>Ertragsgutschrift Roche (netto)</t>
+  </si>
+  <si>
+    <t>Ertragsgutschrift Nestlé (netto)</t>
+  </si>
+  <si>
+    <t>Ertragsgutschrift Fuchs (netto)</t>
+  </si>
+  <si>
+    <t>Storno Ertragsgutschrift Nestlé</t>
+  </si>
+  <si>
+    <t>Ertragsgutschrift Nestlé neu (netto)</t>
+  </si>
+  <si>
+    <t>Ertragsgutschrift Reckitt (netto)</t>
+  </si>
+  <si>
+    <t>Steuererstattung (Übertrag GS-OPS TAX QUEST)</t>
+  </si>
+  <si>
+    <t>Zinsen Tagesgeld Q2 (netto)</t>
+  </si>
+  <si>
+    <t>Zinsen Tagesgeld Q3 (netto)</t>
+  </si>
+  <si>
+    <t>Zinsen Tagesgeld Q4 (netto)</t>
+  </si>
+  <si>
+    <t>Korrigiert 20.10.2026: exakte Centbeträge aus den Finanzreporten; Tagesgeldzinsen Q1, Q3, Q4 ergänzt (bisher nur Q2).</t>
   </si>
   <si>
     <t>Trauerredner</t>
@@ -203,15 +210,9 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10.5"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -247,9 +248,9 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,7 +430,7 @@
         <v>46058</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="13.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -494,22 +495,26 @@
       <c r="A17" t="s">
         <v>13</v>
       </c>
-      <c r="B17">
-        <v>1413</v>
+      <c r="B17" s="3">
+        <f>'Ertrag comdirect 2025'!B23</f>
+        <v>1517.63</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="2">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4">
         <f>SUM(B15:B18)</f>
-        <v>3707.41</v>
+        <v>3812.04</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23">
         <v>12502.3</v>
@@ -517,41 +522,42 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B24">
         <v>-7787.65</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>13</v>
       </c>
-      <c r="B25">
-        <v>1413</v>
+      <c r="B25" s="3">
+        <f>'Ertrag comdirect 2025'!B23</f>
+        <v>1517.63</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" s="2">
+        <v>20</v>
+      </c>
+      <c r="B27" s="4">
         <f>SUM(B23:B26)</f>
-        <v>6127.65</v>
+        <v>6232.28</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Aptos,Standard"&amp;K0000ff Internal&amp;1#_x005F_x000D_&amp;"Times New Roman,Standard"&amp;12&amp;K000000&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12Seite &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Aptos,Standard"&amp;K0000ff Internal&amp;1#_x000D_&amp;"Times New Roman,Standard"&amp;12 &amp;K000000&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12 Seite &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -569,24 +575,24 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="3">
         <v>23548.63</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="3">
         <v>-6558.25</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2">
         <v>3458.18</v>
@@ -594,7 +600,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3">
         <v>3874.27</v>
@@ -604,7 +610,7 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B4" s="4"/>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4">
         <v>3460.27</v>
@@ -613,14 +619,14 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5">
         <f>SUM(B1:B4)</f>
         <v>16990.38</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5">
         <v>3903.26</v>
@@ -634,13 +640,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8">
         <v>18442.41</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E8">
         <v>3874.27</v>
@@ -648,13 +654,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9">
         <v>-5940.11</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E9">
         <v>3913.38</v>
@@ -662,7 +668,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E10">
         <f>SUM(E8:E9)</f>
@@ -674,7 +680,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12">
         <f>SUM(B8:B11)</f>
@@ -1244,12 +1250,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
@@ -1295,7 +1301,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>10848</v>
@@ -1339,7 +1345,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4">
         <v>25099</v>
@@ -1383,7 +1389,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>3915</v>
@@ -1427,7 +1433,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6">
         <v>51751</v>
@@ -1471,110 +1477,148 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>45748</v>
-      </c>
-      <c r="B10">
-        <v>273</v>
+        <v>45747</v>
+      </c>
+      <c r="B10" s="3">
+        <v>33.89</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>45772</v>
-      </c>
-      <c r="B11">
-        <v>278</v>
+        <v>45748</v>
+      </c>
+      <c r="B11" s="3">
+        <v>273.02</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>45789</v>
-      </c>
-      <c r="B12">
-        <v>294</v>
+        <v>45772</v>
+      </c>
+      <c r="B12" s="3">
+        <v>278.7</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>45804</v>
-      </c>
-      <c r="B13">
-        <v>-278</v>
+        <v>45789</v>
+      </c>
+      <c r="B13" s="3">
+        <v>294.87</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>45805</v>
-      </c>
-      <c r="B14">
-        <v>278</v>
+        <v>45804</v>
+      </c>
+      <c r="B14" s="3">
+        <v>-278.7</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>45807</v>
-      </c>
-      <c r="B15">
-        <v>198</v>
+        <v>45805</v>
+      </c>
+      <c r="B15" s="3">
+        <v>278.7</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <v>45838</v>
-      </c>
-      <c r="B16">
-        <v>34</v>
+        <v>45807</v>
+      </c>
+      <c r="B16" s="3">
+        <v>198.27</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>45831</v>
       </c>
-      <c r="B17">
-        <v>204</v>
+      <c r="B17" s="3">
+        <v>204.23</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
+        <v>45838</v>
+      </c>
+      <c r="B18" s="3">
+        <v>33.950000000000003</v>
+      </c>
+      <c r="C18" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>45919</v>
       </c>
-      <c r="B18">
-        <v>132</v>
-      </c>
-      <c r="C18" t="s">
-        <v>39</v>
+      <c r="B19" s="3">
+        <v>132.66999999999999</v>
+      </c>
+      <c r="C19" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="A20" s="1">
+        <v>45930</v>
+      </c>
+      <c r="B20" s="3">
+        <v>33.99</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>46022</v>
+      </c>
+      <c r="B21" s="3">
+        <v>34.04</v>
+      </c>
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>10</v>
       </c>
-      <c r="B20">
-        <f>SUM(B10:B19)</f>
-        <v>1413</v>
+      <c r="B23" s="3">
+        <f>SUM(B10:B21)</f>
+        <v>1517.63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1593,7 +1637,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="B1">
         <v>603</v>
@@ -1601,7 +1645,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="B2">
         <v>843.4</v>
@@ -1609,7 +1653,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="B3">
         <v>5478.75</v>
@@ -1625,8 +1669,8 @@
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12Seite &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12 &amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12 Seite &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>